<commit_message>
Update reference Excel files for signed balance fix
Regenerate all reference Excel files to reflect the corrected balance
calculation that preserves signed amounts. The key changes:

- Balance sheet rows now sorted by signed values (not absolute)
- Income entry balances now correctly reflect positive amounts received
- Member ordering in balance sheets updated accordingly

All tests now pass (20/20).

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tricount_extractor/tests/data/expected_results/custom_category_trip_8.xlsx
+++ b/tricount_extractor/tests/data/expected_results/custom_category_trip_8.xlsx
@@ -952,7 +952,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alice</t>
+          <t>Bob</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -965,7 +965,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bob</t>
+          <t>Alice</t>
         </is>
       </c>
       <c r="C3" t="n">

</xml_diff>